<commit_message>
update: adds xlsx test for DATABASE functions
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DMIN_DMAX_DAVERAGE_DSUM_DCOUNT_DGET.xlsx
+++ b/xlsx/tests/calc_tests/DMIN_DMAX_DAVERAGE_DSUM_DCOUNT_DGET.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29512"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F14C7538-B2B9-48A6-BC82-F25E1134C3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{483B1BA9-FE9E-4293-B67F-0E931C76EC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DATABASE" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="88">
   <si>
     <t>Region</t>
   </si>
@@ -58,18 +58,6 @@
     <t>Contractor</t>
   </si>
   <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>One</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Numbers</t>
-  </si>
-  <si>
     <t>East</t>
   </si>
   <si>
@@ -82,15 +70,6 @@
     <t>Widget</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-  </si>
-  <si>
     <t>West</t>
   </si>
   <si>
@@ -100,39 +79,21 @@
     <t>Gadget</t>
   </si>
   <si>
-    <t>Caracas</t>
-  </si>
-  <si>
     <t>Cara</t>
   </si>
   <si>
     <t>Q2</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>South</t>
   </si>
   <si>
     <t>Dan</t>
   </si>
   <si>
-    <t>BERLIN</t>
-  </si>
-  <si>
     <t>Ella</t>
   </si>
   <si>
-    <t>BB</t>
-  </si>
-  <si>
-    <t>aa</t>
-  </si>
-  <si>
     <t>Frank</t>
   </si>
   <si>
@@ -142,48 +103,24 @@
     <t>Gizmo</t>
   </si>
   <si>
-    <t>balpha</t>
-  </si>
-  <si>
     <t>North</t>
   </si>
   <si>
     <t>Gina</t>
   </si>
   <si>
-    <t>Berlino</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
     <t>Hank</t>
   </si>
   <si>
-    <t>Aa</t>
-  </si>
-  <si>
-    <t>Valencia</t>
-  </si>
-  <si>
     <t>Ivy</t>
   </si>
   <si>
     <t>Q4</t>
   </si>
   <si>
-    <t>Montreal</t>
-  </si>
-  <si>
     <t>Jake</t>
   </si>
   <si>
-    <t>aaa</t>
-  </si>
-  <si>
-    <t>Berlín</t>
-  </si>
-  <si>
     <t>Revnu</t>
   </si>
   <si>
@@ -223,13 +160,7 @@
     <t>WEST</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>&lt;&gt;a</t>
-  </si>
-  <si>
-    <t>&gt;-1</t>
+    <t>???</t>
   </si>
   <si>
     <t>DMIN</t>
@@ -328,48 +259,6 @@
     <t>Field as a number (9, outside of range)</t>
   </si>
   <si>
-    <t>Wildcard (*)</t>
-  </si>
-  <si>
-    <t>Column TRUE, boolean (= 'a')</t>
-  </si>
-  <si>
-    <t>Column true, string (&lt;&gt;'a')</t>
-  </si>
-  <si>
-    <t>Column number (1 could also be true)</t>
-  </si>
-  <si>
-    <t>Cone 'One' (there are two of them)</t>
-  </si>
-  <si>
-    <t>The one with Berlin</t>
-  </si>
-  <si>
-    <t>Numbers and cast bools</t>
-  </si>
-  <si>
-    <t>The same as number 1, but column is by index, not name</t>
-  </si>
-  <si>
-    <t>Counts all numbers in column P</t>
-  </si>
-  <si>
-    <t>Counts all numbers in column index 1</t>
-  </si>
-  <si>
-    <t>Counts all numbers in column "1"</t>
-  </si>
-  <si>
-    <t>Counts all numbers in column TRUE (boolean)</t>
-  </si>
-  <si>
-    <t>Counts all numbers in clumn "true"</t>
-  </si>
-  <si>
-    <t>Doesn't work as it takes as an index</t>
-  </si>
-  <si>
     <t>Rgn</t>
   </si>
   <si>
@@ -382,7 +271,10 @@
     <t>J*</t>
   </si>
   <si>
-    <t>&gt;11/1/2024</t>
+    <t>&gt;01/11/2024</t>
+  </si>
+  <si>
+    <t>????</t>
   </si>
   <si>
     <t>"=400"</t>
@@ -401,15 +293,6 @@
   </si>
   <si>
     <t>Date invalid condition</t>
-  </si>
-  <si>
-    <t>=DGET(A1:G11,F1,L16:L17)</t>
-  </si>
-  <si>
-    <t>Date valid condition</t>
-  </si>
-  <si>
-    <t>&lt;= 11/1/2024 could be 11 January or 1 November. This fails also in Excel</t>
   </si>
   <si>
     <t>Text Patterns (multiple matches)</t>
@@ -422,7 +305,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,6 +337,13 @@
       <name val="Arial"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
@@ -461,7 +351,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -480,14 +370,8 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -616,26 +500,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -688,7 +557,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -724,37 +594,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -970,7 +816,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1009"/>
+  <dimension ref="A1:Z1008"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="7" max="7" width="21.28515625" bestFit="1" customWidth="1"/>
@@ -978,532 +824,301 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="57" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="58" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="58" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="58" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="58" t="b">
+    </row>
+    <row r="2" spans="1:26">
+      <c r="A2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="5">
+        <v>120</v>
+      </c>
+      <c r="F2" s="6">
+        <v>12000</v>
+      </c>
+      <c r="G2" s="7">
+        <v>45306</v>
+      </c>
+      <c r="H2" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="J1" s="59">
+    </row>
+    <row r="3" spans="1:26">
+      <c r="A3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="5">
+        <v>80</v>
+      </c>
+      <c r="F3" s="6">
+        <v>9600</v>
+      </c>
+      <c r="G3" s="7">
+        <v>45324</v>
+      </c>
+      <c r="H3" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8"/>
+    </row>
+    <row r="4" spans="1:26">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="5">
+        <v>200</v>
+      </c>
+      <c r="F4" s="6">
+        <v>20000</v>
+      </c>
+      <c r="G4" s="7">
+        <v>45392</v>
+      </c>
+      <c r="H4" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="K1" s="58" t="s">
+      <c r="J4" s="8"/>
+    </row>
+    <row r="5" spans="1:26">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="5">
+        <v>150</v>
+      </c>
+      <c r="F5" s="6">
+        <v>15000</v>
+      </c>
+      <c r="G5" s="7">
+        <v>45369</v>
+      </c>
+      <c r="H5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="8"/>
+    </row>
+    <row r="6" spans="1:26">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="5">
+        <v>50</v>
+      </c>
+      <c r="F6" s="6">
+        <v>6000</v>
+      </c>
+      <c r="G6" s="7">
+        <v>45434</v>
+      </c>
+      <c r="H6" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8"/>
+    </row>
+    <row r="7" spans="1:26">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="58">
-        <f>1/3</f>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="M1" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" s="58" t="s">
+      <c r="B7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="5">
+        <v>300</v>
+      </c>
+      <c r="F7" s="6">
+        <v>30000</v>
+      </c>
+      <c r="G7" s="7">
+        <v>45481</v>
+      </c>
+      <c r="H7" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" spans="1:26">
+      <c r="A8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:26">
-      <c r="A2" s="60" t="s">
+      <c r="E8" s="5">
+        <v>100</v>
+      </c>
+      <c r="F8" s="6">
+        <v>11000</v>
+      </c>
+      <c r="G8" s="7">
+        <v>45503</v>
+      </c>
+      <c r="H8" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" spans="1:26">
+      <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="60" t="s">
+      <c r="B9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="5">
+        <v>400</v>
+      </c>
+      <c r="F9" s="6">
+        <v>38000</v>
+      </c>
+      <c r="G9" s="7">
+        <v>45515</v>
+      </c>
+      <c r="H9" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" spans="1:26">
+      <c r="A10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="60">
-        <v>120</v>
-      </c>
-      <c r="F2" s="61">
-        <v>12000</v>
-      </c>
-      <c r="G2" s="62">
-        <v>45306</v>
-      </c>
-      <c r="H2" s="61" t="b">
+      <c r="E10" s="5">
+        <v>250</v>
+      </c>
+      <c r="F10" s="6">
+        <v>24000</v>
+      </c>
+      <c r="G10" s="7">
+        <v>45571</v>
+      </c>
+      <c r="H10" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="I2" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61" t="s">
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="61">
+      <c r="B11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="11">
+        <v>200</v>
+      </c>
+      <c r="F11" s="12">
+        <v>19800</v>
+      </c>
+      <c r="G11" s="13">
+        <v>45621</v>
+      </c>
+      <c r="H11" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="M2" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="N2" s="61"/>
-      <c r="O2" s="61" t="s">
-        <v>18</v>
-      </c>
-      <c r="P2" s="61" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26">
-      <c r="A3" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="60" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="60" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="60">
-        <v>80</v>
-      </c>
-      <c r="F3" s="61">
-        <v>9600</v>
-      </c>
-      <c r="G3" s="62">
-        <v>45324</v>
-      </c>
-      <c r="H3" s="61" t="b">
-        <v>0</v>
-      </c>
-      <c r="I3" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" s="61">
-        <v>1</v>
-      </c>
-      <c r="M3" s="61"/>
-      <c r="N3" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" s="61" t="s">
-        <v>22</v>
-      </c>
-      <c r="P3" s="61" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26">
-      <c r="A4" s="60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="60">
-        <v>200</v>
-      </c>
-      <c r="F4" s="61">
-        <v>20000</v>
-      </c>
-      <c r="G4" s="62">
-        <v>45392</v>
-      </c>
-      <c r="H4" s="61" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="61" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="61" t="s">
-        <v>26</v>
-      </c>
-      <c r="K4" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="L4" s="61">
-        <v>1</v>
-      </c>
-      <c r="M4" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="N4" s="61"/>
-      <c r="O4" s="61" t="s">
-        <v>18</v>
-      </c>
-      <c r="P4" s="61">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26">
-      <c r="A5" s="60" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="60" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="60">
-        <v>150</v>
-      </c>
-      <c r="F5" s="61">
-        <v>15000</v>
-      </c>
-      <c r="G5" s="62">
-        <v>45369</v>
-      </c>
-      <c r="H5" s="61" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="61" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5" s="61"/>
-      <c r="K5" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="L5" s="61">
-        <v>1</v>
-      </c>
-      <c r="M5" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="N5" s="61"/>
-      <c r="O5" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="P5" s="61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26">
-      <c r="A6" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="60" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="60">
-        <v>50</v>
-      </c>
-      <c r="F6" s="61">
-        <v>6000</v>
-      </c>
-      <c r="G6" s="62">
-        <v>45434</v>
-      </c>
-      <c r="H6" s="61" t="b">
-        <v>0</v>
-      </c>
-      <c r="I6" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="61" t="s">
-        <v>31</v>
-      </c>
-      <c r="K6" s="61">
-        <v>12</v>
-      </c>
-      <c r="L6" s="61">
-        <v>1</v>
-      </c>
-      <c r="M6" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="N6" s="61"/>
-      <c r="O6" s="61" t="str">
-        <f>" Berlin"</f>
-        <v xml:space="preserve"> Berlin</v>
-      </c>
-      <c r="P6" s="61" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26">
-      <c r="A7" s="60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="60">
-        <v>300</v>
-      </c>
-      <c r="F7" s="61">
-        <v>30000</v>
-      </c>
-      <c r="G7" s="62">
-        <v>45481</v>
-      </c>
-      <c r="H7" s="61" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="61" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J7" s="61" t="s">
-        <v>36</v>
-      </c>
-      <c r="K7" s="61">
-        <v>1</v>
-      </c>
-      <c r="L7" s="61">
-        <v>1</v>
-      </c>
-      <c r="M7" s="61"/>
-      <c r="N7" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="O7" s="61" t="str">
-        <f>" Berlin "</f>
-        <v xml:space="preserve"> Berlin </v>
-      </c>
-      <c r="P7" s="61"/>
-    </row>
-    <row r="8" spans="1:26">
-      <c r="A8" s="60" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="60" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="60">
-        <v>100</v>
-      </c>
-      <c r="F8" s="61">
-        <v>11000</v>
-      </c>
-      <c r="G8" s="62">
-        <v>45503</v>
-      </c>
-      <c r="H8" s="61" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L8" s="61">
-        <v>2</v>
-      </c>
-      <c r="M8" s="61"/>
-      <c r="N8" s="61"/>
-      <c r="O8" s="61" t="s">
-        <v>39</v>
-      </c>
-      <c r="P8" s="61" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26">
-      <c r="A9" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="60" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="60">
-        <v>400</v>
-      </c>
-      <c r="F9" s="61">
-        <v>38000</v>
-      </c>
-      <c r="G9" s="62">
-        <v>45515</v>
-      </c>
-      <c r="H9" s="61" t="b">
-        <v>0</v>
-      </c>
-      <c r="I9" s="61">
-        <v>23</v>
-      </c>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="L9" s="61">
-        <v>1</v>
-      </c>
-      <c r="M9" s="61" t="s">
-        <v>42</v>
-      </c>
-      <c r="N9" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="O9" s="61" t="s">
-        <v>43</v>
-      </c>
-      <c r="P9" s="61"/>
-    </row>
-    <row r="10" spans="1:26">
-      <c r="A10" s="60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="60" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="60" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="60">
-        <v>250</v>
-      </c>
-      <c r="F10" s="61">
-        <v>24000</v>
-      </c>
-      <c r="G10" s="62">
-        <v>45571</v>
-      </c>
-      <c r="H10" s="61" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="61">
-        <v>455</v>
-      </c>
-      <c r="J10" s="61">
-        <v>23</v>
-      </c>
-      <c r="K10" s="61" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" s="61">
-        <v>12</v>
-      </c>
-      <c r="M10" s="61" t="str">
-        <f>" aa"</f>
-        <v xml:space="preserve"> aa</v>
-      </c>
-      <c r="N10" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="O10" s="61" t="s">
-        <v>46</v>
-      </c>
-      <c r="P10" s="61">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26">
-      <c r="A11" s="60" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="60" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="60" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="63">
-        <v>200</v>
-      </c>
-      <c r="F11" s="61">
-        <v>19800</v>
-      </c>
-      <c r="G11" s="62">
-        <v>45621</v>
-      </c>
-      <c r="H11" s="61" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="61">
-        <v>2</v>
-      </c>
-      <c r="J11" s="61"/>
-      <c r="K11" s="61" t="e">
-        <f>1/0</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L11" s="61"/>
-      <c r="M11" s="61" t="s">
-        <v>48</v>
-      </c>
-      <c r="N11" s="61"/>
-      <c r="O11" s="61" t="s">
-        <v>49</v>
-      </c>
-      <c r="P11" s="61"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:26">
-      <c r="F12" s="55">
-        <f>SUM(F2:F11)</f>
-        <v>185400</v>
-      </c>
       <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:26">
@@ -1599,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="O14" s="18" t="s">
         <v>1</v>
@@ -1618,53 +1233,53 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="19" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="J15" s="26" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="K15" s="27"/>
       <c r="L15" s="27" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="M15" s="27" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="N15" s="27"/>
       <c r="O15" s="27" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:26">
       <c r="D16" s="24" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H16" s="8"/>
     </row>
@@ -1745,7 +1360,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="J19" s="15" t="s">
         <v>0</v>
@@ -1776,26 +1391,26 @@
         <v>1</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E20" s="19"/>
       <c r="F20" s="19" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="H20" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="I20" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="I20" s="19" t="s">
-        <v>19</v>
-      </c>
       <c r="J20" s="19" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="K20" s="19" t="str">
         <f t="shared" ref="K20:L20" si="0">"East"</f>
@@ -1806,16 +1421,16 @@
         <v>East</v>
       </c>
       <c r="M20" s="19" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N20" s="19" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="O20" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="P20" s="27" t="s">
-        <v>63</v>
+        <v>8</v>
+      </c>
+      <c r="P20" s="19" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1825,73 +1440,13 @@
       <c r="J22" s="8"/>
     </row>
     <row r="23" spans="1:16">
-      <c r="I23" s="14">
-        <v>29</v>
-      </c>
-      <c r="J23" s="14">
-        <v>30</v>
-      </c>
-      <c r="K23" s="14">
-        <v>31</v>
-      </c>
-      <c r="L23" s="14">
-        <v>32</v>
-      </c>
-      <c r="M23" s="14">
-        <v>33</v>
-      </c>
-      <c r="N23" s="14">
-        <v>34</v>
-      </c>
-      <c r="O23" s="14">
-        <v>35</v>
-      </c>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" spans="1:16">
-      <c r="I24" s="18" t="b">
-        <v>1</v>
-      </c>
-      <c r="J24" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="K24" s="56">
-        <v>1</v>
-      </c>
-      <c r="L24" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="M24" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="N24" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="O24" s="18" t="s">
-        <v>0</v>
-      </c>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" spans="1:16">
-      <c r="I25" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="K25" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="L25" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="M25" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="N25" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="O25" s="27" t="s">
-        <v>12</v>
-      </c>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" spans="1:16">
       <c r="J26" s="8"/>
@@ -1899,19 +1454,19 @@
     <row r="27" spans="1:16">
       <c r="A27" s="28"/>
       <c r="B27" s="29" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="F27" s="29" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="J27" s="8"/>
     </row>
@@ -1919,28 +1474,28 @@
       <c r="A28" s="28">
         <v>1</v>
       </c>
-      <c r="B28" s="30">
+      <c r="B28" s="31">
         <f>DMIN($A$1:$G$11,$F$1,A14:A15)</f>
         <v>12000</v>
       </c>
-      <c r="C28" s="30">
+      <c r="C28" s="31">
         <f>DMAX($A$1:$G$11,$F$1,A14:A15)</f>
         <v>30000</v>
       </c>
-      <c r="D28" s="30">
+      <c r="D28" s="31">
         <f>DAVERAGE($A$1:$G$11,$F$1,A14:A15)</f>
         <v>21500</v>
       </c>
-      <c r="E28" s="30">
+      <c r="E28" s="31">
         <f>DSUM($A$1:$G$11,$F$1,A14:A15)</f>
         <v>86000</v>
       </c>
-      <c r="F28" s="30">
+      <c r="F28" s="31">
         <f>DCOUNT($A$1:$G$11,$F$1,A14:A15)</f>
         <v>4</v>
       </c>
       <c r="G28" s="28" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="J28" s="8"/>
     </row>
@@ -1948,28 +1503,28 @@
       <c r="A29" s="28">
         <v>2</v>
       </c>
-      <c r="B29" s="30">
+      <c r="B29" s="31">
         <f>DMIN($A$1:$G$11,$E$1,B14:C15)</f>
         <v>120</v>
       </c>
-      <c r="C29" s="30">
+      <c r="C29" s="31">
         <f>DMAX($A$1:$G$11,E1,B14:C15)</f>
         <v>200</v>
       </c>
-      <c r="D29" s="30">
+      <c r="D29" s="31">
         <f>DAVERAGE($A$1:$G$11,E1,B14:C15)</f>
         <v>160</v>
       </c>
-      <c r="E29" s="30">
+      <c r="E29" s="31">
         <f>DSUM($A$1:$G$11,E1,B14:C15)</f>
         <v>320</v>
       </c>
-      <c r="F29" s="30">
+      <c r="F29" s="31">
         <f>DCOUNT($A$1:$G$11,E1,B14:C15)</f>
         <v>2</v>
       </c>
       <c r="G29" s="28" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J29" s="8"/>
     </row>
@@ -1977,86 +1532,92 @@
       <c r="A30" s="28">
         <v>3</v>
       </c>
-      <c r="B30" s="30">
+      <c r="B30" s="31">
         <f>DMIN(A1:G11,F1,D14:E16)</f>
         <v>6000</v>
       </c>
-      <c r="C30" s="30">
+      <c r="C30" s="31">
         <f>DMAX($A$1:$G$11,F1,D14:E16)</f>
         <v>12000</v>
       </c>
-      <c r="D30" s="30">
+      <c r="D30" s="31">
         <f>DAVERAGE($A$1:$G$11,F1,D14:E16)</f>
         <v>9000</v>
       </c>
-      <c r="E30" s="30">
+      <c r="E30" s="31">
         <f>DSUM($A$1:$G$11,F1,D14:E16)</f>
         <v>18000</v>
       </c>
-      <c r="F30" s="30">
+      <c r="F30" s="31">
         <f>DCOUNT($A$1:$G$11,F1,D14:E16)</f>
         <v>2</v>
       </c>
       <c r="G30" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="J30" s="8"/>
+        <v>50</v>
+      </c>
+      <c r="J30" s="31">
+        <f>DMIN($A$1:$G$11,$F$1,$B$14:$B$15)</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="28">
         <v>4</v>
       </c>
-      <c r="B31" s="30">
+      <c r="B31" s="31">
         <f>DMIN(A1:G11,F1,F14:F15)</f>
         <v>12000</v>
       </c>
-      <c r="C31" s="30">
+      <c r="C31" s="31">
         <f>DMAX(A1:G11,F1,F14:F15)</f>
         <v>38000</v>
       </c>
-      <c r="D31" s="30">
+      <c r="D31" s="31">
         <f>DAVERAGE(A1:G11,F1,F14:F15)</f>
         <v>22685.714285714286</v>
       </c>
-      <c r="E31" s="30">
+      <c r="E31" s="31">
         <f>DSUM(A1:G11,F1,F14:F15)</f>
         <v>158800</v>
       </c>
-      <c r="F31" s="30">
+      <c r="F31" s="31">
         <f>DCOUNT(A1:G11,F1,F14:F15)</f>
         <v>7</v>
       </c>
       <c r="G31" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="J31" s="8"/>
+        <v>51</v>
+      </c>
+      <c r="J31" s="31">
+        <f>DMIN($A$1:$G$11,$F$1,$B$14:$B$15)</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="28">
         <v>5</v>
       </c>
-      <c r="B32" s="30">
+      <c r="B32" s="31">
         <f>DMIN(A1:G11,F1,G14:H15)</f>
         <v>12000</v>
       </c>
-      <c r="C32" s="30">
+      <c r="C32" s="31">
         <f>DMAX(A1:G11,F1,G14:H15)</f>
         <v>19800</v>
       </c>
-      <c r="D32" s="30">
+      <c r="D32" s="31">
         <f>DAVERAGE(A1:G11,F1,G14:H15)</f>
         <v>15600</v>
       </c>
-      <c r="E32" s="30">
+      <c r="E32" s="31">
         <f>DSUM(A1:G11,F1,G14:H15)</f>
         <v>46800</v>
       </c>
-      <c r="F32" s="30">
+      <c r="F32" s="31">
         <f>DCOUNT(A1:G11,F1,G14:H15)</f>
         <v>3</v>
       </c>
       <c r="G32" s="28" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="J32" s="8"/>
     </row>
@@ -2064,28 +1625,28 @@
       <c r="A33" s="28">
         <v>6</v>
       </c>
-      <c r="B33" s="30">
+      <c r="B33" s="31">
         <f>DMIN(A1:G11,F1,I14:I15)</f>
         <v>11000</v>
       </c>
-      <c r="C33" s="30">
+      <c r="C33" s="31">
         <f>DMAX(A1:G11,F1,I14:I15)</f>
         <v>38000</v>
       </c>
-      <c r="D33" s="30">
+      <c r="D33" s="31">
         <f>DAVERAGE(A1:G11,F1,I14:I15)</f>
         <v>24560</v>
       </c>
-      <c r="E33" s="30">
+      <c r="E33" s="31">
         <f>DSUM(A1:G11,F1,I14:I15)</f>
         <v>122800</v>
       </c>
-      <c r="F33" s="30">
+      <c r="F33" s="31">
         <f>DCOUNT(A1:G11,F1,I14:I15)</f>
         <v>5</v>
       </c>
       <c r="G33" s="28" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="J33" s="8"/>
     </row>
@@ -2093,28 +1654,28 @@
       <c r="A34" s="28">
         <v>7</v>
       </c>
-      <c r="B34" s="30">
+      <c r="B34" s="31">
         <f>DMIN(A1:G11,F1,J14:J15)</f>
         <v>6000</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C34" s="31">
         <f>DMAX(A1:G11,F1,J14:J15)</f>
         <v>30000</v>
       </c>
-      <c r="D34" s="30">
+      <c r="D34" s="31">
         <f>DAVERAGE(A1:G11,F1,J14:J15)</f>
         <v>17400</v>
       </c>
-      <c r="E34" s="30">
+      <c r="E34" s="31">
         <f>DSUM(A1:G11,F1,J14:J15)</f>
         <v>69600</v>
       </c>
-      <c r="F34" s="30">
+      <c r="F34" s="31">
         <f>DCOUNT(A1:G11,F1,J14:J15)</f>
         <v>4</v>
       </c>
       <c r="G34" s="28" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="J34" s="8"/>
     </row>
@@ -2122,28 +1683,28 @@
       <c r="A35" s="28">
         <v>8</v>
       </c>
-      <c r="B35" s="30">
+      <c r="B35" s="31">
         <f>DMIN(A1:G11,F1,K14:K15)</f>
         <v>6000</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="31">
         <f>DMAX(A1:G11,F1,K14:K15)</f>
         <v>38000</v>
       </c>
-      <c r="D35" s="30">
+      <c r="D35" s="31">
         <f>DAVERAGE(A1:G11,F1,K14:K15)</f>
         <v>18540</v>
       </c>
-      <c r="E35" s="30">
+      <c r="E35" s="31">
         <f>DSUM(A1:G11,F1,K14:K15)</f>
         <v>185400</v>
       </c>
-      <c r="F35" s="30">
+      <c r="F35" s="31">
         <f>DCOUNT(A1:G11,F1,K14:K15)</f>
         <v>10</v>
       </c>
       <c r="G35" s="28" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="J35" s="8"/>
     </row>
@@ -2151,28 +1712,28 @@
       <c r="A36" s="28">
         <v>9</v>
       </c>
-      <c r="B36" s="30">
+      <c r="B36" s="31">
         <f>DMIN(A1:G11,F1,L14:L15)</f>
         <v>0</v>
       </c>
-      <c r="C36" s="30">
+      <c r="C36" s="31">
         <f>DMAX(A1:G11,F1,L14:L15)</f>
         <v>0</v>
       </c>
-      <c r="D36" s="30" t="e">
+      <c r="D36" s="31" t="e">
         <f>DAVERAGE(A1:G11,F1,L14:L15)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E36" s="30">
+      <c r="E36" s="31">
         <f>DSUM(A1:G11,F1,L14:L15)</f>
         <v>0</v>
       </c>
-      <c r="F36" s="30">
+      <c r="F36" s="31">
         <f>DCOUNT(A1:G11,F1,L14:L15)</f>
         <v>0</v>
       </c>
       <c r="G36" s="28" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="J36" s="8"/>
     </row>
@@ -2180,28 +1741,28 @@
       <c r="A37" s="28">
         <v>10</v>
       </c>
-      <c r="B37" s="30">
+      <c r="B37" s="31">
         <f>DMIN(A1:G11,F1,M14:M15)</f>
         <v>0</v>
       </c>
-      <c r="C37" s="30">
+      <c r="C37" s="31">
         <f>DMAX(A1:G11,F1,M14:M15)</f>
         <v>0</v>
       </c>
-      <c r="D37" s="30" t="e">
+      <c r="D37" s="31" t="e">
         <f>DAVERAGE(A1:G11,F1,M14:M15)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E37" s="30">
+      <c r="E37" s="31">
         <f>DSUM(A1:G11,F1,M14:M15)</f>
         <v>0</v>
       </c>
-      <c r="F37" s="30">
+      <c r="F37" s="31">
         <f>DCOUNT(A1:G11,F1,M14:M15)</f>
         <v>0</v>
       </c>
       <c r="G37" s="28" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="J37" s="8"/>
     </row>
@@ -2209,28 +1770,28 @@
       <c r="A38" s="28">
         <v>11</v>
       </c>
-      <c r="B38" s="30">
+      <c r="B38" s="31">
         <f>DMIN(A1:G11,F1,N14:N15)</f>
         <v>6000</v>
       </c>
-      <c r="C38" s="30">
+      <c r="C38" s="31">
         <f>DMAX(A1:G11,F1,N14:N15)</f>
         <v>38000</v>
       </c>
-      <c r="D38" s="30">
+      <c r="D38" s="31">
         <f>DAVERAGE(A1:G11,F1,N14:N15)</f>
         <v>18540</v>
       </c>
-      <c r="E38" s="30">
+      <c r="E38" s="31">
         <f>DSUM(A1:G11,F1,N14:N15)</f>
         <v>185400</v>
       </c>
-      <c r="F38" s="30">
+      <c r="F38" s="31">
         <f>DCOUNT(A1:G11,F1,N14:N15)</f>
         <v>10</v>
       </c>
       <c r="G38" s="28" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="J38" s="8"/>
     </row>
@@ -2238,28 +1799,28 @@
       <c r="A39" s="28">
         <v>12</v>
       </c>
-      <c r="B39" s="30">
+      <c r="B39" s="31">
         <f>DMIN(A1:G11,F1,O14:O15)</f>
         <v>30000</v>
       </c>
-      <c r="C39" s="30">
+      <c r="C39" s="31">
         <f>DMAX(A1:G11,F1,O14:O15)</f>
         <v>38000</v>
       </c>
-      <c r="D39" s="30">
+      <c r="D39" s="31">
         <f>DAVERAGE(A1:G11,F1,O14:O15)</f>
         <v>34000</v>
       </c>
-      <c r="E39" s="30">
+      <c r="E39" s="31">
         <f>DSUM(A1:G11,F1,O14:O15)</f>
         <v>68000</v>
       </c>
-      <c r="F39" s="30">
+      <c r="F39" s="31">
         <f>DCOUNT(A1:G11,F1,O14:O15)</f>
         <v>2</v>
       </c>
       <c r="G39" s="28" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="J39" s="8"/>
     </row>
@@ -2267,28 +1828,28 @@
       <c r="A40" s="28">
         <v>13</v>
       </c>
-      <c r="B40" s="30">
+      <c r="B40" s="31">
         <f>DMIN(A1:H11,F1,A19:A20)</f>
         <v>12000</v>
       </c>
-      <c r="C40" s="30">
+      <c r="C40" s="31">
         <f>DMAX(A1:H11,F1,A19:A20)</f>
         <v>30000</v>
       </c>
-      <c r="D40" s="30">
+      <c r="D40" s="31">
         <f>DAVERAGE(A1:H11,F1,A19:A20)</f>
         <v>20133.333333333332</v>
       </c>
-      <c r="E40" s="30">
+      <c r="E40" s="31">
         <f>DSUM(A1:H11,F1,A19:A20)</f>
         <v>120800</v>
       </c>
-      <c r="F40" s="30">
+      <c r="F40" s="31">
         <f>DCOUNT(A1:H11,F1,A19:A20)</f>
         <v>6</v>
       </c>
       <c r="G40" s="28" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="J40" s="8"/>
     </row>
@@ -2296,28 +1857,28 @@
       <c r="A41" s="28">
         <v>14</v>
       </c>
-      <c r="B41" s="30">
+      <c r="B41" s="31">
         <f>DMIN(A1:H11,F1,B19:B20)</f>
         <v>0</v>
       </c>
-      <c r="C41" s="30">
+      <c r="C41" s="31">
         <f>DMAX(A1:H11,F1,B19:B20)</f>
         <v>0</v>
       </c>
-      <c r="D41" s="30" t="e">
+      <c r="D41" s="31" t="e">
         <f>DAVERAGE(A1:H11,F1,B19:B20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E41" s="30">
+      <c r="E41" s="31">
         <f>DSUM(A1:H11,F1,B19:B20)</f>
         <v>0</v>
       </c>
-      <c r="F41" s="30">
+      <c r="F41" s="31">
         <f>DCOUNT(A1:H11,F1,B19:B20)</f>
         <v>0</v>
       </c>
       <c r="G41" s="28" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="J41" s="8"/>
     </row>
@@ -2325,28 +1886,28 @@
       <c r="A42" s="28">
         <v>15</v>
       </c>
-      <c r="B42" s="30">
+      <c r="B42" s="31">
         <f>DMIN(A1:H11,F1,C19:C20)</f>
         <v>0</v>
       </c>
-      <c r="C42" s="30">
+      <c r="C42" s="31">
         <f>DMAX(A1:H11,F1,C19:C20)</f>
         <v>0</v>
       </c>
-      <c r="D42" s="30" t="e">
+      <c r="D42" s="31" t="e">
         <f>DAVERAGE(A1:H11,F1,C19:C20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E42" s="30">
+      <c r="E42" s="31">
         <f>DSUM(A1:H11,F1,C19:C20)</f>
         <v>0</v>
       </c>
-      <c r="F42" s="30">
+      <c r="F42" s="31">
         <f>DCOUNT(A1:H11,F1,C19:C20)</f>
         <v>0</v>
       </c>
       <c r="G42" s="28" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="J42" s="8"/>
     </row>
@@ -2354,28 +1915,28 @@
       <c r="A43" s="28">
         <v>16</v>
       </c>
-      <c r="B43" s="30" t="e">
+      <c r="B43" s="31" t="e">
         <f>DMIN(A1:H1,F1,D19:D20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C43" s="30" t="e">
+      <c r="C43" s="31" t="e">
         <f>DMAX(A1:H1,F1,D19:D20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D43" s="30" t="e">
+      <c r="D43" s="31" t="e">
         <f>DAVERAGE(A1:H1,F1,D19:D20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E43" s="30" t="e">
+      <c r="E43" s="31" t="e">
         <f>DSUM(A1:H1,F1,D19:D20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F43" s="30" t="e">
+      <c r="F43" s="31" t="e">
         <f>DCOUNT(A1:H1,F1,D19:D20)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G43" s="28" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="J43" s="8"/>
     </row>
@@ -2383,28 +1944,28 @@
       <c r="A44" s="28">
         <v>17</v>
       </c>
-      <c r="B44" s="30" t="e">
+      <c r="B44" s="31" t="e">
         <f>DMIN(A1:H1,A22,E19:E20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C44" s="30" t="e">
+      <c r="C44" s="31" t="e">
         <f>DMAX(A1:H1,A22,E19:E20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D44" s="30" t="e">
+      <c r="D44" s="31" t="e">
         <f>DAVERAGE(A1:H1,A22,E19:E20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E44" s="30" t="e">
+      <c r="E44" s="31" t="e">
         <f>DSUM(A1:H1,A22,E19:E20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F44" s="30" t="e">
+      <c r="F44" s="31" t="e">
         <f>DCOUNT(A1:H1,A22,E19:E20)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G44" s="28" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="J44" s="8"/>
     </row>
@@ -2412,28 +1973,28 @@
       <c r="A45" s="28">
         <v>18</v>
       </c>
-      <c r="B45" s="30">
+      <c r="B45" s="31">
         <f>DMIN(A1:H11,F1,F19:F20)</f>
         <v>0</v>
       </c>
-      <c r="C45" s="30">
+      <c r="C45" s="31">
         <f>DMAX(A1:H11,F1,F19:F20)</f>
         <v>0</v>
       </c>
-      <c r="D45" s="30" t="e">
+      <c r="D45" s="31" t="e">
         <f>DAVERAGE(A1:H11,F1,F19:F20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E45" s="30">
+      <c r="E45" s="31">
         <f>DSUM(A1:H11,F1,F19:F20)</f>
         <v>0</v>
       </c>
-      <c r="F45" s="30">
+      <c r="F45" s="31">
         <f>DCOUNT(A1:H11,F1,F19:F20)</f>
         <v>0</v>
       </c>
       <c r="G45" s="28" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="J45" s="8"/>
     </row>
@@ -2441,28 +2002,28 @@
       <c r="A46" s="28">
         <v>19</v>
       </c>
-      <c r="B46" s="30">
+      <c r="B46" s="31">
         <f>DMIN(A1:H11,F1,G19:G20)</f>
         <v>0</v>
       </c>
-      <c r="C46" s="30">
+      <c r="C46" s="31">
         <f>DMAX(A1:H11,F1,G19:G20)</f>
         <v>0</v>
       </c>
-      <c r="D46" s="30" t="e">
+      <c r="D46" s="31" t="e">
         <f>DAVERAGE(A1:H11,F1,G19:G20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E46" s="30">
+      <c r="E46" s="31">
         <f>DSUM(A1:H11,F1,G19:G20)</f>
         <v>0</v>
       </c>
-      <c r="F46" s="30">
+      <c r="F46" s="31">
         <f>DCOUNT(A1:H11,F1,G19:G20)</f>
         <v>0</v>
       </c>
       <c r="G46" s="28" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="J46" s="8"/>
     </row>
@@ -2470,28 +2031,28 @@
       <c r="A47" s="28">
         <v>20</v>
       </c>
-      <c r="B47" s="30" t="e">
+      <c r="B47" s="31" t="e">
         <f>DMIN(A2:H11,F1,H19:H20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C47" s="30" t="e">
+      <c r="C47" s="31" t="e">
         <f>DMAX(A2:H11,F1,H19:H20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D47" s="30" t="e">
+      <c r="D47" s="31" t="e">
         <f>DAVERAGE(A2:H11,F1,H19:H20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E47" s="30" t="e">
+      <c r="E47" s="31" t="e">
         <f>DSUM(A2:H11,F1,H19:H20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F47" s="30" t="e">
+      <c r="F47" s="31" t="e">
         <f>DCOUNT(A2:H11,F1,H19:H20)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G47" s="28" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="J47" s="8"/>
     </row>
@@ -2499,28 +2060,28 @@
       <c r="A48" s="28">
         <v>21</v>
       </c>
-      <c r="B48" s="30">
+      <c r="B48" s="31">
         <f>DMIN(A1:H11,F1,I19:I20)</f>
         <v>6000</v>
       </c>
-      <c r="C48" s="30">
+      <c r="C48" s="31">
         <f>DMAX(A1:H11,F1,I19:I20)</f>
         <v>38000</v>
       </c>
-      <c r="D48" s="30">
+      <c r="D48" s="31">
         <f>DAVERAGE(A1:H11,F1,I19:I20)</f>
         <v>17866.666666666668</v>
       </c>
-      <c r="E48" s="30">
+      <c r="E48" s="31">
         <f>DSUM(A1:H11,F1,I19:I20)</f>
         <v>53600</v>
       </c>
-      <c r="F48" s="30">
+      <c r="F48" s="31">
         <f>DCOUNT(A1:H11,F1,I19:I20)</f>
         <v>3</v>
       </c>
       <c r="G48" s="28" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="J48" s="8"/>
     </row>
@@ -2528,28 +2089,28 @@
       <c r="A49" s="28">
         <v>22</v>
       </c>
-      <c r="B49" s="30">
+      <c r="B49" s="31">
         <f>DMIN(A1:H11,F1,J19:J20)</f>
         <v>6000</v>
       </c>
-      <c r="C49" s="30">
+      <c r="C49" s="31">
         <f>DMAX(A1:H11,F1,J19:J20)</f>
         <v>38000</v>
       </c>
-      <c r="D49" s="30">
+      <c r="D49" s="31">
         <f>DAVERAGE(A1:H11,F1,J19:J20)</f>
         <v>17866.666666666668</v>
       </c>
-      <c r="E49" s="30">
+      <c r="E49" s="31">
         <f>DSUM(A1:H11,F1,J19:J20)</f>
         <v>53600</v>
       </c>
-      <c r="F49" s="30">
+      <c r="F49" s="31">
         <f>DCOUNT(A1:H11,F1,J19:J20)</f>
         <v>3</v>
       </c>
       <c r="G49" s="28" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="J49" s="8"/>
     </row>
@@ -2557,28 +2118,28 @@
       <c r="A50" s="28">
         <v>23</v>
       </c>
-      <c r="B50" s="30">
+      <c r="B50" s="31">
         <f>DMIN(A1:H11,F1,K19:K20)</f>
         <v>12000</v>
       </c>
-      <c r="C50" s="30">
+      <c r="C50" s="31">
         <f>DMAX(A1:H11,F1,K19:K20)</f>
         <v>30000</v>
       </c>
-      <c r="D50" s="30">
+      <c r="D50" s="31">
         <f>DAVERAGE(A1:H11,F1,K19:K20)</f>
         <v>21500</v>
       </c>
-      <c r="E50" s="30">
+      <c r="E50" s="31">
         <f>DSUM(A1:H11,F1,K19:K20)</f>
         <v>86000</v>
       </c>
-      <c r="F50" s="30">
+      <c r="F50" s="31">
         <f>DCOUNT(A1:H11,F1,K19:K20)</f>
         <v>4</v>
       </c>
       <c r="G50" s="28" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="J50" s="8"/>
     </row>
@@ -2586,28 +2147,28 @@
       <c r="A51" s="28">
         <v>24</v>
       </c>
-      <c r="B51" s="30">
+      <c r="B51" s="31">
         <f>DMIN(A1:H11,F1,L19:L20)</f>
         <v>0</v>
       </c>
-      <c r="C51" s="30">
+      <c r="C51" s="31">
         <f>DMAX(A1:H11,F1,L19:L20)</f>
         <v>0</v>
       </c>
-      <c r="D51" s="30" t="e">
+      <c r="D51" s="31" t="e">
         <f>DAVERAGE(A1:H11,F1,L19:L20)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E51" s="30">
+      <c r="E51" s="31">
         <f>DSUM(A1:H11,F1,L19:L20)</f>
         <v>0</v>
       </c>
-      <c r="F51" s="30">
+      <c r="F51" s="31">
         <f>DCOUNT(A1:H11,F1,L19:L20)</f>
         <v>0</v>
       </c>
       <c r="G51" s="28" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="J51" s="8"/>
     </row>
@@ -2615,28 +2176,28 @@
       <c r="A52" s="28">
         <v>25</v>
       </c>
-      <c r="B52" s="30">
+      <c r="B52" s="31">
         <f>DMIN(A1:H11,6,M19:M20)</f>
         <v>12000</v>
       </c>
-      <c r="C52" s="30">
+      <c r="C52" s="31">
         <f>DMAX(A1:H11,6,M19:M20)</f>
         <v>30000</v>
       </c>
-      <c r="D52" s="30">
+      <c r="D52" s="31">
         <f>DAVERAGE(A1:H11,6,M19:M20)</f>
         <v>21500</v>
       </c>
-      <c r="E52" s="30">
+      <c r="E52" s="31">
         <f>DSUM(A1:H11,6,M19:M20)</f>
         <v>86000</v>
       </c>
-      <c r="F52" s="30">
+      <c r="F52" s="31">
         <f>DCOUNT(A1:H11,6,M19:M20)</f>
         <v>4</v>
       </c>
       <c r="G52" s="28" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="J52" s="8"/>
     </row>
@@ -2644,28 +2205,28 @@
       <c r="A53" s="28">
         <v>25</v>
       </c>
-      <c r="B53" s="30" t="e">
+      <c r="B53" s="31" t="e">
         <f>DMIN(A1:H11,0,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C53" s="30" t="e">
+      <c r="C53" s="31" t="e">
         <f>DMAX(A1:H11,0,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D53" s="30" t="e">
+      <c r="D53" s="31" t="e">
         <f>DAVERAGE(A1:H11,0,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E53" s="30" t="e">
+      <c r="E53" s="31" t="e">
         <f>DSUM(A1:H11,0,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F53" s="30" t="e">
+      <c r="F53" s="31" t="e">
         <f>DCOUNT(A1:H11,0,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G53" s="28" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="J53" s="8"/>
     </row>
@@ -2673,357 +2234,117 @@
       <c r="A54" s="28">
         <v>25</v>
       </c>
-      <c r="B54" s="30" t="e">
+      <c r="B54" s="31" t="e">
         <f>DMIN(A1:H11,9,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C54" s="30" t="e">
+      <c r="C54" s="31" t="e">
         <f>DMAX(A1:H11,9,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D54" s="30" t="e">
+      <c r="D54" s="31" t="e">
         <f>DAVERAGE(A1:H11,9,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E54" s="30" t="e">
+      <c r="E54" s="31" t="e">
         <f>DSUM(A1:H11,9,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F54" s="30" t="e">
+      <c r="F54" s="31" t="e">
         <f>DCOUNT(A1:H11,9,M19:M20)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G54" s="28" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="J54" s="8"/>
     </row>
     <row r="55" spans="1:10">
-      <c r="A55" s="28">
-        <v>28</v>
-      </c>
-      <c r="B55" s="30">
-        <f>DMIN(A1:H11,F1,P19:P20)</f>
-        <v>6000</v>
-      </c>
-      <c r="C55" s="30">
-        <f>DMAX(A1:H11,F1,P19:P20)</f>
-        <v>38000</v>
-      </c>
-      <c r="D55" s="30">
-        <f>DAVERAGE(A1:H11,F1,P19:P20)</f>
-        <v>18540</v>
-      </c>
-      <c r="E55" s="30">
-        <f>DSUM(A1:H11,F1,P19:P20)</f>
-        <v>185400</v>
-      </c>
-      <c r="F55" s="30">
-        <f>DCOUNT(A1:H11,F1,P19:P20)</f>
-        <v>10</v>
-      </c>
-      <c r="G55" s="28" t="s">
-        <v>98</v>
-      </c>
+      <c r="F55" s="30"/>
+      <c r="G55" s="32"/>
       <c r="J55" s="8"/>
     </row>
     <row r="56" spans="1:10">
-      <c r="A56" s="28">
-        <v>29</v>
-      </c>
-      <c r="B56" s="30">
-        <f>DMIN(A1:K11,F1,I24:I25)</f>
-        <v>6000</v>
-      </c>
-      <c r="C56" s="30">
-        <f>DMAX(A1:K11,F1,I24:I25)</f>
-        <v>20000</v>
-      </c>
-      <c r="D56" s="30">
-        <f>DAVERAGE(A1:K11,F1,I24:I25)</f>
-        <v>13250</v>
-      </c>
-      <c r="E56" s="30">
-        <f>DSUM(A1:K11,F1,I24:I25)</f>
-        <v>53000</v>
-      </c>
-      <c r="F56" s="30">
-        <f>DCOUNT(A1:K11,F1,I24:I25)</f>
-        <v>4</v>
-      </c>
-      <c r="G56" s="31" t="s">
-        <v>99</v>
-      </c>
+      <c r="F56" s="30"/>
+      <c r="G56" s="32"/>
       <c r="J56" s="8"/>
     </row>
     <row r="57" spans="1:10">
-      <c r="A57" s="28">
-        <v>30</v>
-      </c>
-      <c r="B57" s="30">
-        <f>DMIN(A1:K11,F1,J24:J25)</f>
-        <v>9600</v>
-      </c>
-      <c r="C57" s="30">
-        <f>DMAX(A1:K11,F1,J24:J25)</f>
-        <v>38000</v>
-      </c>
-      <c r="D57" s="30">
-        <f>DAVERAGE(A1:K11,F1,J24:J25)</f>
-        <v>22066.666666666668</v>
-      </c>
-      <c r="E57" s="30">
-        <f>DSUM(A1:K11,F1,J24:J25)</f>
-        <v>132400</v>
-      </c>
-      <c r="F57" s="30">
-        <f>DCOUNT(A1:K11,F1,J24:J25)</f>
-        <v>6</v>
-      </c>
-      <c r="G57" s="31" t="s">
-        <v>100</v>
-      </c>
+      <c r="F57" s="30"/>
       <c r="J57" s="8"/>
     </row>
     <row r="58" spans="1:10">
-      <c r="A58" s="28">
-        <v>31</v>
-      </c>
-      <c r="B58" s="30">
-        <f>DMIN(A1:O11,F1,K24:K25)</f>
-        <v>6000</v>
-      </c>
-      <c r="C58" s="30">
-        <f>DMAX(A1:O11,F1,K24:K25)</f>
-        <v>30000</v>
-      </c>
-      <c r="D58" s="30">
-        <f>DAVERAGE(A1:O11,F1,K24:K25)</f>
-        <v>16400</v>
-      </c>
-      <c r="E58" s="30">
-        <f>DSUM(A1:O11,F1,K24:K25)</f>
-        <v>65600</v>
-      </c>
-      <c r="F58" s="30">
-        <f>DCOUNT(A1:O11,F1,K24:K25)</f>
-        <v>4</v>
-      </c>
-      <c r="G58" t="s">
-        <v>101</v>
-      </c>
+      <c r="F58" s="30"/>
       <c r="J58" s="8"/>
     </row>
     <row r="59" spans="1:10">
-      <c r="A59" s="28">
-        <v>32</v>
-      </c>
-      <c r="B59" s="30">
-        <f>DMIN(A1:O11,F1,L24:L25)</f>
-        <v>6000</v>
-      </c>
-      <c r="C59" s="30">
-        <f>DMAX(A1:O11,F1,L24:L25)</f>
-        <v>38000</v>
-      </c>
-      <c r="D59" s="30">
-        <f>DAVERAGE(A1:O11,F1,L24:L25)</f>
-        <v>21266.666666666668</v>
-      </c>
-      <c r="E59" s="30">
-        <f>DSUM(A1:O11,F1,L24:L25)</f>
-        <v>63800</v>
-      </c>
-      <c r="F59" s="30">
-        <f>DCOUNT(A1:O11,F1,L24:L25)</f>
-        <v>3</v>
-      </c>
-      <c r="G59" t="s">
-        <v>102</v>
-      </c>
+      <c r="F59" s="30"/>
       <c r="J59" s="8"/>
     </row>
     <row r="60" spans="1:10">
-      <c r="A60" s="28">
-        <v>33</v>
-      </c>
-      <c r="B60" s="30">
-        <f>DMIN(A1:O11,F1,M24:M25)</f>
-        <v>11000</v>
-      </c>
-      <c r="C60" s="30">
-        <f>DMAX(A1:O11,F1,M24:M25)</f>
-        <v>20000</v>
-      </c>
-      <c r="D60" s="30">
-        <f>DAVERAGE(A1:O11,F1,M24:M25)</f>
-        <v>14500</v>
-      </c>
-      <c r="E60" s="30">
-        <f>DSUM(A1:O11,F1,M24:M25)</f>
-        <v>58000</v>
-      </c>
-      <c r="F60" s="30">
-        <f>DCOUNT(A1:O11,F1,M24:M25)</f>
-        <v>4</v>
-      </c>
-      <c r="G60" t="s">
-        <v>103</v>
-      </c>
+      <c r="F60" s="30"/>
       <c r="J60" s="8"/>
     </row>
     <row r="61" spans="1:10">
-      <c r="A61" s="28">
-        <v>34</v>
-      </c>
-      <c r="B61" s="30">
-        <f>DMIN(A1:P11,P1,N24:N25)</f>
-        <v>1</v>
-      </c>
-      <c r="C61" s="30">
-        <f>DMAX(A1:P11,P1,N24:N25)</f>
-        <v>7</v>
-      </c>
-      <c r="D61" s="30">
-        <f>DAVERAGE(A1:P11,P1,N24:N25)</f>
-        <v>4</v>
-      </c>
-      <c r="E61" s="30">
-        <f>DSUM(A1:P11,P1,N24:N25)</f>
-        <v>8</v>
-      </c>
-      <c r="F61" s="30">
-        <f>DCOUNT(A1:P11,P1,N24:N25)</f>
-        <v>2</v>
-      </c>
-      <c r="G61" t="s">
-        <v>104</v>
-      </c>
+      <c r="F61" s="30"/>
       <c r="J61" s="8"/>
     </row>
     <row r="62" spans="1:10">
-      <c r="A62">
-        <v>35</v>
-      </c>
-      <c r="B62" s="30">
-        <f>DMIN($A$1:$G$11,6.7,O24:O25)</f>
-        <v>12000</v>
-      </c>
-      <c r="C62" s="30">
-        <f>DMAX($A$1:$G$11,6.1,O24:O25)</f>
-        <v>30000</v>
-      </c>
-      <c r="D62" s="30" t="e">
-        <f>DAVERAGE($A$1:$G$11,-1,O24:O25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E62" s="30">
-        <f>DSUM($A$1:$G$11,6.99,O24:O25)</f>
-        <v>86000</v>
-      </c>
-      <c r="F62" s="30">
-        <f>DCOUNT($A$1:$G$11,6,O24:O25)</f>
-        <v>4</v>
-      </c>
-      <c r="G62" t="s">
-        <v>105</v>
-      </c>
+      <c r="F62" s="30"/>
       <c r="J62" s="8"/>
     </row>
     <row r="63" spans="1:10">
-      <c r="F63" s="30">
-        <f>DCOUNT($A$1:$P$11,"Numbers",P19:P20)</f>
-        <v>3</v>
-      </c>
-      <c r="G63" t="s">
-        <v>106</v>
-      </c>
       <c r="J63" s="8"/>
     </row>
     <row r="64" spans="1:10">
-      <c r="F64" s="30">
-        <f>DCOUNT($A$1:$P$11,1,P19:P20)</f>
-        <v>0</v>
-      </c>
-      <c r="G64" t="s">
-        <v>107</v>
-      </c>
       <c r="J64" s="8"/>
     </row>
-    <row r="65" spans="6:10">
-      <c r="F65" s="30">
-        <f>DCOUNT($A$1:$P$11,"1",P19:P20)</f>
-        <v>1</v>
-      </c>
-      <c r="G65" t="s">
-        <v>108</v>
-      </c>
+    <row r="65" spans="10:10">
       <c r="J65" s="8"/>
     </row>
-    <row r="66" spans="6:10">
-      <c r="F66" s="30">
-        <f>DCOUNT($A$1:$P$11,TRUE,P2:P19)</f>
-        <v>0</v>
-      </c>
-      <c r="G66" t="s">
-        <v>109</v>
-      </c>
+    <row r="66" spans="10:10">
       <c r="J66" s="8"/>
     </row>
-    <row r="67" spans="6:10">
-      <c r="F67" s="30">
-        <f>DCOUNT($A$1:$P$11,"true",P2:P19)</f>
-        <v>3</v>
-      </c>
-      <c r="G67" t="s">
-        <v>110</v>
-      </c>
+    <row r="67" spans="10:10">
       <c r="J67" s="8"/>
     </row>
-    <row r="68" spans="6:10">
-      <c r="F68" s="30" t="e">
-        <f>DCOUNT($A$1:$P$11,1/3,P2:P19)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G68" t="s">
-        <v>111</v>
-      </c>
+    <row r="68" spans="10:10">
       <c r="J68" s="8"/>
     </row>
-    <row r="69" spans="6:10">
+    <row r="69" spans="10:10">
       <c r="J69" s="8"/>
     </row>
-    <row r="70" spans="6:10">
+    <row r="70" spans="10:10">
       <c r="J70" s="8"/>
     </row>
-    <row r="71" spans="6:10">
+    <row r="71" spans="10:10">
       <c r="J71" s="8"/>
     </row>
-    <row r="72" spans="6:10">
+    <row r="72" spans="10:10">
       <c r="J72" s="8"/>
     </row>
-    <row r="73" spans="6:10">
+    <row r="73" spans="10:10">
       <c r="J73" s="8"/>
     </row>
-    <row r="74" spans="6:10">
+    <row r="74" spans="10:10">
       <c r="J74" s="8"/>
     </row>
-    <row r="75" spans="6:10">
+    <row r="75" spans="10:10">
       <c r="J75" s="8"/>
     </row>
-    <row r="76" spans="6:10">
+    <row r="76" spans="10:10">
       <c r="J76" s="8"/>
     </row>
-    <row r="77" spans="6:10">
+    <row r="77" spans="10:10">
       <c r="J77" s="8"/>
     </row>
-    <row r="78" spans="6:10">
+    <row r="78" spans="10:10">
       <c r="J78" s="8"/>
     </row>
-    <row r="79" spans="6:10">
+    <row r="79" spans="10:10">
       <c r="J79" s="8"/>
     </row>
-    <row r="80" spans="6:10">
+    <row r="80" spans="10:10">
       <c r="J80" s="8"/>
     </row>
     <row r="81" spans="10:10">
@@ -5809,9 +5130,6 @@
     </row>
     <row r="1008" spans="10:10">
       <c r="J1008" s="8"/>
-    </row>
-    <row r="1009" spans="10:10">
-      <c r="J1009" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -5823,7 +5141,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q56"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
@@ -5858,16 +5176,16 @@
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E2" s="5">
         <v>120</v>
@@ -5884,16 +5202,16 @@
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="E3" s="5">
         <v>80</v>
@@ -5910,16 +5228,16 @@
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E4" s="5">
         <v>200</v>
@@ -5936,16 +5254,16 @@
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E5" s="5">
         <v>150</v>
@@ -5962,16 +5280,16 @@
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>30</v>
-      </c>
       <c r="C6" s="5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E6" s="5">
         <v>50</v>
@@ -5988,16 +5306,16 @@
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="E7" s="5">
         <v>300</v>
@@ -6014,16 +5332,16 @@
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E8" s="5">
         <v>100</v>
@@ -6040,16 +5358,16 @@
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E9" s="5">
         <v>400</v>
@@ -6066,16 +5384,16 @@
     </row>
     <row r="10" spans="1:17" ht="15" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E10" s="5">
         <v>250</v>
@@ -6092,16 +5410,16 @@
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1">
       <c r="A11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>45</v>
-      </c>
       <c r="D11" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E11" s="11">
         <v>200</v>
@@ -6116,7 +5434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="39" customFormat="1" ht="15" customHeight="1">
+    <row r="13" spans="1:17" s="40" customFormat="1" ht="15" customHeight="1">
       <c r="A13" s="14">
         <v>1</v>
       </c>
@@ -6129,13 +5447,13 @@
       <c r="D13" s="14">
         <v>4</v>
       </c>
-      <c r="E13" s="39">
+      <c r="E13" s="40">
         <v>5</v>
       </c>
-      <c r="G13" s="39">
+      <c r="G13" s="40">
         <v>6</v>
       </c>
-      <c r="I13" s="39">
+      <c r="I13" s="40">
         <v>7</v>
       </c>
       <c r="J13" s="14">
@@ -6159,29 +5477,29 @@
       </c>
       <c r="Q13"/>
     </row>
-    <row r="14" spans="1:17" s="40" customFormat="1" ht="15" customHeight="1">
-      <c r="A14" s="32" t="s">
+    <row r="14" spans="1:17" s="41" customFormat="1" ht="15" customHeight="1">
+      <c r="A14" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="32" t="s">
-        <v>112</v>
-      </c>
-      <c r="E14" s="32" t="s">
+      <c r="D14" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="F14" s="34" t="s">
+      <c r="F14" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="H14" s="34" t="s">
+      <c r="H14" s="35" t="s">
         <v>3</v>
       </c>
       <c r="I14" s="18" t="s">
@@ -6206,63 +5524,63 @@
         <v>0</v>
       </c>
       <c r="P14" s="18" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="Q14"/>
     </row>
-    <row r="15" spans="1:17" s="35" customFormat="1" ht="15" customHeight="1">
-      <c r="A15" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="D15" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="E15" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="H15" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="45">
+    <row r="15" spans="1:17" s="36" customFormat="1" ht="15" customHeight="1">
+      <c r="A15" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="46">
         <v>100</v>
       </c>
-      <c r="J15" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="K15" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="L15" s="49">
+      <c r="J15" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="L15" s="50">
         <v>45474</v>
       </c>
-      <c r="M15" s="45" t="s">
-        <v>115</v>
-      </c>
-      <c r="N15" s="48"/>
-      <c r="O15" s="45" t="s">
-        <v>56</v>
-      </c>
-      <c r="P15" s="45"/>
+      <c r="M15" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="N15" s="49"/>
+      <c r="O15" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="P15" s="46"/>
       <c r="Q15"/>
     </row>
-    <row r="16" spans="1:17" s="35" customFormat="1" ht="15" customHeight="1">
-      <c r="G16" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>35</v>
+    <row r="16" spans="1:17" s="36" customFormat="1" ht="15" customHeight="1">
+      <c r="G16" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>22</v>
       </c>
       <c r="L16" s="18" t="s">
         <v>6</v>
@@ -6272,15 +5590,15 @@
       </c>
       <c r="Q16"/>
     </row>
-    <row r="17" spans="1:15" ht="15" customHeight="1">
-      <c r="L17" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="M17" s="45" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="15" customHeight="1">
+    <row r="17" spans="1:13" ht="15" customHeight="1">
+      <c r="L17" s="50" t="s">
+        <v>79</v>
+      </c>
+      <c r="M17" s="46" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="15" customHeight="1">
       <c r="L18" s="14">
         <v>10</v>
       </c>
@@ -6288,7 +5606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="15" customHeight="1">
+    <row r="19" spans="1:13" ht="15" customHeight="1">
       <c r="A19" s="14">
         <v>15</v>
       </c>
@@ -6317,7 +5635,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="15" customHeight="1">
+    <row r="20" spans="1:13" ht="15" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>7</v>
       </c>
@@ -6334,7 +5652,7 @@
         <v>6</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="G20" s="15" t="s">
         <v>0</v>
@@ -6345,7 +5663,7 @@
       </c>
       <c r="I20" s="18"/>
     </row>
-    <row r="21" spans="1:15" ht="15" customHeight="1">
+    <row r="21" spans="1:13" ht="15" customHeight="1">
       <c r="A21" s="19" t="b">
         <v>1</v>
       </c>
@@ -6353,19 +5671,19 @@
         <v>1</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="H21" s="19" t="str">
         <f t="shared" ref="H21:I21" si="0">"East"</f>
@@ -6376,408 +5694,377 @@
         <v>East</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="15" customHeight="1">
+    <row r="23" spans="1:13" ht="15" customHeight="1">
       <c r="A23" s="28"/>
       <c r="B23" s="29" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="C23" s="28"/>
-      <c r="O23" s="64"/>
-    </row>
-    <row r="24" spans="1:15" ht="15" customHeight="1">
+    </row>
+    <row r="24" spans="1:13" ht="15" customHeight="1">
       <c r="A24" s="28">
         <v>1</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="31">
         <f>DGET($A$1:$H$11,$F$1,A14:A15)</f>
         <v>11000</v>
       </c>
-      <c r="C24" s="50" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="15" customHeight="1">
+      <c r="C24" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15" customHeight="1">
       <c r="A25" s="28">
         <v>2</v>
       </c>
-      <c r="B25" s="30" t="e">
+      <c r="B25" s="31" t="e">
         <f>DGET($A$1:$H$11,$F$1,B14:B15)</f>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="50" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="15" customHeight="1">
+      <c r="C25" s="28" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15" customHeight="1">
       <c r="A26" s="28">
         <v>3</v>
       </c>
-      <c r="B26" s="30" t="e">
+      <c r="B26" s="31" t="e">
         <f>DGET($A$1:$H$11,$F$1,C14:C15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C26" s="50" t="s">
-        <v>121</v>
-      </c>
-      <c r="E26" s="28"/>
-    </row>
-    <row r="27" spans="1:15" ht="15" customHeight="1">
+      <c r="C26" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15" customHeight="1">
       <c r="A27" s="28">
         <v>4</v>
       </c>
-      <c r="B27" s="30" t="e">
+      <c r="B27" s="31" t="e">
         <f>DGET($A$1:$H$11,$F$1,D14:D15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C27" s="50" t="s">
-        <v>81</v>
-      </c>
-      <c r="E27" s="30">
-        <f>DCOUNT($A$1:$H$11,$F$1,D14:D15)</f>
-        <v>0</v>
+      <c r="C27" s="28" t="s">
+        <v>58</v>
       </c>
       <c r="F27" s="28"/>
     </row>
-    <row r="28" spans="1:15" ht="15" customHeight="1">
+    <row r="28" spans="1:13" ht="15" customHeight="1">
       <c r="A28" s="28">
         <v>5</v>
       </c>
-      <c r="B28" s="30">
+      <c r="B28" s="31">
         <f>DGET($A$1:$H$11,$F$1,E14:F15)</f>
         <v>11000</v>
       </c>
-      <c r="C28" s="50" t="s">
-        <v>72</v>
-      </c>
-      <c r="E28" s="28"/>
+      <c r="C28" s="28" t="s">
+        <v>49</v>
+      </c>
       <c r="F28" s="28"/>
     </row>
-    <row r="29" spans="1:15" ht="15" customHeight="1">
+    <row r="29" spans="1:13" ht="15" customHeight="1">
       <c r="A29" s="28">
         <v>6</v>
       </c>
-      <c r="B29" s="30">
+      <c r="B29" s="31">
         <f>DGET($A$1:$H$11,$F$1,G14:H16)</f>
         <v>11000</v>
       </c>
-      <c r="C29" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="E29" s="28"/>
+      <c r="C29" s="28" t="s">
+        <v>50</v>
+      </c>
       <c r="F29" s="28"/>
     </row>
-    <row r="30" spans="1:15" ht="15" customHeight="1">
+    <row r="30" spans="1:13" ht="15" customHeight="1">
       <c r="A30" s="28">
         <v>7</v>
       </c>
-      <c r="B30" s="30">
+      <c r="B30" s="31">
         <f>DGET($A$1:$H$11,$F$1,I14:I15)</f>
         <v>11000</v>
       </c>
-      <c r="C30" s="50" t="s">
-        <v>74</v>
+      <c r="C30" s="28" t="s">
+        <v>51</v>
       </c>
       <c r="F30" s="28"/>
     </row>
-    <row r="31" spans="1:15" ht="15" customHeight="1">
+    <row r="31" spans="1:13" ht="15" customHeight="1">
       <c r="A31" s="28">
         <v>8</v>
       </c>
-      <c r="B31" s="30">
+      <c r="B31" s="31">
         <f>DGET(A1:G11,F1,J14:K15)</f>
         <v>38000</v>
       </c>
-      <c r="C31" s="50" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="15" customHeight="1">
+      <c r="C31" s="28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="15" customHeight="1">
       <c r="A32" s="28">
         <v>9</v>
       </c>
-      <c r="B32" s="30" t="e">
+      <c r="B32" s="31" t="e">
         <f>DGET(A1:G11,F1,L14:L15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C32" s="50" t="s">
-        <v>122</v>
+      <c r="C32" s="28" t="s">
+        <v>86</v>
       </c>
       <c r="F32" s="28"/>
     </row>
     <row r="33" spans="1:6" ht="15" customHeight="1">
-      <c r="A33" s="53">
-        <v>10</v>
-      </c>
-      <c r="B33" s="65" t="s">
-        <v>123</v>
-      </c>
-      <c r="C33" s="54" t="s">
-        <v>124</v>
-      </c>
-      <c r="E33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F33" s="28"/>
-    </row>
-    <row r="34" spans="1:6" ht="15" customHeight="1">
-      <c r="A34" s="28">
+      <c r="A33" s="28">
         <v>11</v>
       </c>
-      <c r="B34" s="30">
+      <c r="B33" s="31">
         <f>DGET(A1:G11,F1,M14:M15)</f>
         <v>19800</v>
       </c>
-      <c r="C34" s="50" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="15" customHeight="1">
-      <c r="A35" s="28"/>
-      <c r="B35" s="30" t="e">
+      <c r="C33" s="28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15" customHeight="1">
+      <c r="A34" s="28"/>
+      <c r="B34" s="31" t="e">
         <f>DGET(A1:G11,F1,M16:M17)</f>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="50" t="s">
-        <v>126</v>
-      </c>
+      <c r="C34" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="15" customHeight="1">
+      <c r="A35" s="28">
+        <v>12</v>
+      </c>
+      <c r="B35" s="31" t="e">
+        <f>DGET(A1:G11,F1,N14:N15)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C35" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="28"/>
     </row>
     <row r="36" spans="1:6" ht="15" customHeight="1">
       <c r="A36" s="28">
-        <v>12</v>
-      </c>
-      <c r="B36" s="30" t="e">
-        <f>DGET(A1:G11,F1,N14:N15)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C36" s="50" t="s">
-        <v>78</v>
+        <v>13</v>
+      </c>
+      <c r="B36" s="31" t="e">
+        <f>DGET(A1:G11,F1,O14:O15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C36" s="28" t="s">
+        <v>57</v>
       </c>
       <c r="F36" s="28"/>
     </row>
     <row r="37" spans="1:6" ht="15" customHeight="1">
       <c r="A37" s="28">
-        <v>13</v>
-      </c>
-      <c r="B37" s="30" t="e">
-        <f>DGET(A1:G11,F1,O14:O15)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C37" s="50" t="s">
-        <v>80</v>
+        <v>14</v>
+      </c>
+      <c r="B37" s="31" t="e">
+        <f>DGET(A1:G11,F1,P14:P15)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C37" s="28" t="s">
+        <v>58</v>
       </c>
       <c r="F37" s="28"/>
     </row>
     <row r="38" spans="1:6" ht="15" customHeight="1">
       <c r="A38" s="28">
-        <v>14</v>
-      </c>
-      <c r="B38" s="30" t="e">
-        <f>DGET(A1:G11,F1,P14:P15)</f>
+        <v>15</v>
+      </c>
+      <c r="B38" s="31" t="e">
+        <f>DGET(A1:H11,F1,A20:A21)</f>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="50" t="s">
-        <v>81</v>
-      </c>
-      <c r="F38" s="28"/>
+      <c r="C38" s="28" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1">
       <c r="A39" s="28">
-        <v>15</v>
-      </c>
-      <c r="B39" s="30" t="e">
-        <f>DGET(A1:H11,F1,A20:A21)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C39" s="50" t="s">
-        <v>83</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B39" s="31" t="e">
+        <f>DGET(A1:H11,F1,B20:B21)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="F39" s="28"/>
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1">
       <c r="A40" s="28">
-        <v>16</v>
-      </c>
-      <c r="B40" s="30" t="e">
-        <f>DGET(A1:H11,F1,B20:B21)</f>
+        <v>17</v>
+      </c>
+      <c r="B40" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,C20:C21)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C40" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="F40" s="28"/>
+      <c r="C40" s="28" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1">
       <c r="A41" s="28">
-        <v>17</v>
-      </c>
-      <c r="B41" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,C20:C21)</f>
+        <v>1</v>
+      </c>
+      <c r="B41" s="31" t="e">
+        <f>DGET($A$1:$H$1,$F$1,A14:A15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C41" s="50" t="s">
-        <v>85</v>
+      <c r="C41" s="28" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15" customHeight="1">
       <c r="A42" s="28">
         <v>1</v>
       </c>
-      <c r="B42" s="30" t="e">
-        <f>DGET($A$1:$H$1,$F$1,A14:A15)</f>
+      <c r="B42" s="31" t="e">
+        <f>DGET($A$1:$H$11,J3,A14:A15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C42" s="50" t="s">
-        <v>86</v>
-      </c>
+      <c r="C42" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="F42" s="28"/>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1">
       <c r="A43" s="28">
-        <v>1</v>
-      </c>
-      <c r="B43" s="30" t="e">
-        <f>DGET($A$1:$H$11,J3,A14:A15)</f>
+        <v>18</v>
+      </c>
+      <c r="B43" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,D20:D21)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C43" s="50" t="s">
-        <v>94</v>
-      </c>
-      <c r="F43" s="28"/>
+      <c r="C43" s="28" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1">
       <c r="A44" s="28">
-        <v>18</v>
-      </c>
-      <c r="B44" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,D20:D21)</f>
+        <v>19</v>
+      </c>
+      <c r="B44" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,E20:E21)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C44" s="50" t="s">
-        <v>88</v>
+      <c r="C44" s="28" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15" customHeight="1">
       <c r="A45" s="28">
-        <v>19</v>
-      </c>
-      <c r="B45" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,E20:E21)</f>
+        <v>2</v>
+      </c>
+      <c r="B45" s="31" t="e">
+        <f>DGET(A2:$H$11,$F$1,B14:B15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C45" s="50" t="s">
-        <v>89</v>
+      <c r="C45" s="28" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" customHeight="1">
       <c r="A46" s="28">
-        <v>2</v>
-      </c>
-      <c r="B46" s="30" t="e">
-        <f>DGET(A2:$H$11,$F$1,B14:B15)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C46" s="50" t="s">
-        <v>90</v>
+        <v>20</v>
+      </c>
+      <c r="B46" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,F20:F21)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C46" s="28" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1">
       <c r="A47" s="28">
-        <v>20</v>
-      </c>
-      <c r="B47" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,F20:F21)</f>
+        <v>21</v>
+      </c>
+      <c r="B47" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,G20:G21)</f>
         <v>#NUM!</v>
       </c>
-      <c r="C47" s="50" t="s">
-        <v>91</v>
+      <c r="C47" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1">
       <c r="A48" s="28">
-        <v>21</v>
-      </c>
-      <c r="B48" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,G20:G21)</f>
+        <v>22</v>
+      </c>
+      <c r="B48" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,H20:H21)</f>
         <v>#NUM!</v>
       </c>
-      <c r="C48" s="50" t="s">
-        <v>92</v>
+      <c r="C48" s="28" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="15" customHeight="1">
       <c r="A49" s="28">
-        <v>22</v>
-      </c>
-      <c r="B49" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,H20:H21)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C49" s="50" t="s">
-        <v>93</v>
+        <v>23</v>
+      </c>
+      <c r="B49" s="31" t="e">
+        <f>DGET($A$1:$H$11,$F$1,I20:I21)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C49" s="28" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15" customHeight="1">
       <c r="A50" s="28">
-        <v>23</v>
-      </c>
-      <c r="B50" s="30" t="e">
-        <f>DGET($A$1:$H$11,$F$1,I20:I21)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C50" s="50" t="s">
-        <v>94</v>
+        <v>1</v>
+      </c>
+      <c r="B50" s="31">
+        <f>DGET(A1:$H$11,6,$A$14:$A$15)</f>
+        <v>11000</v>
+      </c>
+      <c r="C50" s="28" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="15" customHeight="1">
       <c r="A51" s="28">
         <v>1</v>
       </c>
-      <c r="B51" s="30">
-        <f>DGET(A1:$H$11,6,$A$14:$A$15)</f>
-        <v>11000</v>
-      </c>
-      <c r="C51" s="50" t="s">
-        <v>95</v>
+      <c r="B51" s="31" t="e">
+        <f>DGET(A1:$H$11,0,$A$14:$A$15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C51" s="28" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15" customHeight="1">
       <c r="A52" s="28">
         <v>1</v>
       </c>
-      <c r="B52" s="30" t="e">
-        <f>DGET(A1:$H$11,0,$A$14:$A$15)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C52" s="50" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="15" customHeight="1">
-      <c r="A53" s="28">
-        <v>1</v>
-      </c>
-      <c r="B53" s="30" t="e">
+      <c r="B52" s="31" t="e">
         <f>DGET(A1:$H$11,9,$A$14:$A$15)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C53" s="50" t="s">
-        <v>97</v>
-      </c>
+      <c r="C52" s="28" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="15" customHeight="1">
+      <c r="C53" s="51"/>
     </row>
     <row r="54" spans="1:3" ht="15" customHeight="1">
-      <c r="A54" s="28">
-        <v>27</v>
-      </c>
-      <c r="B54" s="30"/>
-      <c r="C54" s="50"/>
+      <c r="C54" s="51"/>
     </row>
     <row r="55" spans="1:3" ht="15" customHeight="1">
-      <c r="A55" s="28">
-        <v>28</v>
-      </c>
-      <c r="B55" s="30"/>
-      <c r="C55" s="50"/>
-    </row>
-    <row r="56" spans="1:3" ht="15" customHeight="1">
-      <c r="C56" s="51"/>
+      <c r="C55" s="51"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>